<commit_message>
docs(cdc): pre-remplit l'onglet MAINTENANCE avec l'ancien flux existant
Le code contenait deja une implementation Maintenance/demande materiel :
- table demande_materiel + hook useDemandesMateriel
- workflow : en_attente_validation -> validation Sylvain ANTZ ->
  creation tache commande logistique -> demande_de_devis ->
  bon_de_commande_envoye -> ar_recu -> commande_livree -> commande_distribuee
- edge function validate-material-request

J'extrait ce flux dans le CDC pour qu'il soit aligne avec le reste des
modules. Quelques questions restent ouvertes (suppleant Sylvain, motif
refus, plafond budgetaire, reset prod).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CDC/CDC_MODULES.xlsx
+++ b/docs/CDC/CDC_MODULES.xlsx
@@ -8433,7 +8433,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I117"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -8530,7 +8530,7 @@
         <v>Nom metier</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>Maintenance - Demande de materiel</v>
       </c>
       <c r="C6" t="str">
         <v>ex. Maintenance, RH, SMQ</v>
@@ -8541,7 +8541,7 @@
         <v>Code court (URL)</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>maintenance</v>
       </c>
       <c r="C7" t="str">
         <v>ex. maint, rh, smq</v>
@@ -8552,7 +8552,7 @@
         <v>Service responsable</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>Service Maintenance</v>
       </c>
       <c r="C8" t="str">
         <v>equipe traitante</v>
@@ -8563,7 +8563,7 @@
         <v>Manager du service</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>Sylvain ANTZ</v>
       </c>
       <c r="C9" t="str">
         <v>prenom NOM</v>
@@ -8574,7 +8574,7 @@
         <v>Hub projet/dossier ?</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="C10" t="str">
         <v>OUI / NON</v>
@@ -8585,7 +8585,7 @@
         <v>Plusieurs sous-types ?</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="C11" t="str">
         <v>OUI / NON</v>
@@ -8596,7 +8596,7 @@
         <v>Demandeurs autorises</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>techniciens du service maintenance</v>
       </c>
       <c r="C12" t="str">
         <v>tous / managers / services X,Y</v>
@@ -8607,7 +8607,7 @@
         <v>Donnees sensibles ?</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="C13" t="str">
         <v>OUI / NON</v>
@@ -8654,25 +8654,25 @@
         <v>1</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>DEMANDE DE MATERIEL</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>Commande d articles de maintenance</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>logistique apres validation coordinateur</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>Sylvain ANTZ (coordinateur)</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="G17" t="str">
-        <v/>
+        <v>variable selon delai fournisseur</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>date livraison souhaitee</v>
       </c>
     </row>
     <row r="18">
@@ -8832,7 +8832,7 @@
         <v>auto</v>
       </c>
       <c r="G25" t="str">
-        <v>pre-rempli</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -8863,7 +8863,7 @@
         <v>3</v>
       </c>
       <c r="B27" t="str">
-        <v>Description</v>
+        <v>Justification / contexte</v>
       </c>
       <c r="C27" t="str">
         <v>textarea</v>
@@ -8878,7 +8878,7 @@
         <v>demandeur</v>
       </c>
       <c r="G27" t="str">
-        <v/>
+        <v>pour appuyer la validation</v>
       </c>
     </row>
     <row r="28">
@@ -8886,13 +8886,13 @@
         <v>4</v>
       </c>
       <c r="B28" t="str">
-        <v>Pieces jointes</v>
+        <v>Lignes d articles</v>
       </c>
       <c r="C28" t="str">
-        <v>files</v>
+        <v>sub-table</v>
       </c>
       <c r="D28" t="str">
-        <v>NON</v>
+        <v>OUI</v>
       </c>
       <c r="E28" t="str">
         <v>COMMUN</v>
@@ -8901,7 +8901,7 @@
         <v>demandeur</v>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>cf. ligne ci-dessous</v>
       </c>
     </row>
     <row r="29">
@@ -8909,22 +8909,22 @@
         <v>5</v>
       </c>
       <c r="B29" t="str">
-        <v/>
+        <v xml:space="preserve">  - Article (ref)</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>select (catalogue Divalto)</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>OUI</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>COMMUN</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="G29" t="str">
-        <v/>
+        <v>autocomplete sur referentiel articles</v>
       </c>
     </row>
     <row r="30">
@@ -8932,22 +8932,22 @@
         <v>6</v>
       </c>
       <c r="B30" t="str">
-        <v/>
+        <v xml:space="preserve">  - Designation</v>
       </c>
       <c r="C30" t="str">
-        <v/>
+        <v>text</v>
       </c>
       <c r="D30" t="str">
-        <v/>
+        <v>auto</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>COMMUN</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>auto</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>rempli depuis l article</v>
       </c>
     </row>
     <row r="31">
@@ -8955,19 +8955,19 @@
         <v>7</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v xml:space="preserve">  - Quantite</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>number</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>OUI</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>COMMUN</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -8978,22 +8978,22 @@
         <v>8</v>
       </c>
       <c r="B32" t="str">
-        <v/>
+        <v>Date de besoin</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>date</v>
       </c>
       <c r="D32" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>COMMUN</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>optionnel</v>
       </c>
     </row>
     <row r="33">
@@ -9001,22 +9001,22 @@
         <v>9</v>
       </c>
       <c r="B33" t="str">
-        <v/>
+        <v>Pieces jointes</v>
       </c>
       <c r="C33" t="str">
-        <v/>
+        <v>files</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>COMMUN</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="G33" t="str">
-        <v/>
+        <v>photo, plan, devis...</v>
       </c>
     </row>
     <row r="34">
@@ -9043,474 +9043,483 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="str">
+      <c r="A35">
+        <v>11</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="str">
-        <v># Aide types</v>
+      <c r="A36">
+        <v>12</v>
       </c>
       <c r="B36" t="str">
-        <v>text / textarea / number / date / datetime / select / multi-select / bool / files / profile / company / department</v>
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="str">
-        <v># Communs OU prestation</v>
+      <c r="A37">
+        <v>13</v>
       </c>
       <c r="B37" t="str">
-        <v>COMMUN ou nom(s) prestation(s) separes par |</v>
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="str">
+      <c r="A38">
+        <v>14</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>### 4. WORKFLOW (etats et transitions) ###</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v># Aide types</v>
+      </c>
+      <c r="B40" t="str">
+        <v>text / textarea / number / date / datetime / select / multi-select / bool / files / profile / company / department</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v># Communs OU prestation</v>
+      </c>
+      <c r="B41" t="str">
+        <v>COMMUN ou nom(s) prestation(s) separes par |</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>### 4. WORKFLOW (etats et transitions) ###</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
         <v>#</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B44" t="str">
         <v>Statut</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C44" t="str">
         <v>Description</v>
       </c>
-      <c r="D40" t="str">
+      <c r="D44" t="str">
         <v>Qui agit ?</v>
       </c>
-      <c r="E40" t="str">
+      <c r="E44" t="str">
         <v>Statuts suivants</v>
       </c>
-      <c r="F40" t="str">
+      <c r="F44" t="str">
         <v>Action UI (label bouton)</v>
       </c>
-      <c r="G40" t="str">
+      <c r="G44" t="str">
         <v>Effet</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41">
-        <v>1</v>
-      </c>
-      <c r="B41" t="str">
-        <v>soumise</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Demande creee</v>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
-      <c r="E41" t="str">
-        <v/>
-      </c>
-      <c r="F41" t="str">
-        <v/>
-      </c>
-      <c r="G41" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42">
-        <v>2</v>
-      </c>
-      <c r="B42" t="str">
-        <v>affectee</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Affectee a executant</v>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
-      <c r="E42" t="str">
-        <v/>
-      </c>
-      <c r="F42" t="str">
-        <v/>
-      </c>
-      <c r="G42" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="B43" t="str">
-        <v>en_cours</v>
-      </c>
-      <c r="C43" t="str">
-        <v>En cours</v>
-      </c>
-      <c r="D43" t="str">
-        <v/>
-      </c>
-      <c r="E43" t="str">
-        <v/>
-      </c>
-      <c r="F43" t="str">
-        <v/>
-      </c>
-      <c r="G43" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44">
-        <v>4</v>
-      </c>
-      <c r="B44" t="str">
-        <v>a_valider</v>
-      </c>
-      <c r="C44" t="str">
-        <v>Attente validation</v>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
-      <c r="E44" t="str">
-        <v/>
-      </c>
-      <c r="F44" t="str">
-        <v/>
-      </c>
-      <c r="G44" t="str">
-        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B45" t="str">
-        <v>complement_demande</v>
+        <v>en_attente_validation</v>
       </c>
       <c r="C45" t="str">
-        <v>Manque info</v>
+        <v>Demande creee, attente validation coordinateur</v>
       </c>
       <c r="D45" t="str">
-        <v/>
+        <v>Sylvain ANTZ</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>demande_de_devis / refusee</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>Valider / Refuser</v>
       </c>
       <c r="G45" t="str">
-        <v/>
+        <v>a la validation : creation tache commande pour logistique</v>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B46" t="str">
-        <v>realisee</v>
+        <v>demande_de_devis</v>
       </c>
       <c r="C46" t="str">
-        <v>Terminee</v>
+        <v>Logistique cherche fournisseur / devis</v>
       </c>
       <c r="D46" t="str">
-        <v>-</v>
+        <v>logistique</v>
       </c>
       <c r="E46" t="str">
-        <v>-</v>
+        <v>bon_de_commande_envoye</v>
       </c>
       <c r="F46" t="str">
-        <v>-</v>
+        <v>Devis recu</v>
       </c>
       <c r="G46" t="str">
-        <v>terminal</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B47" t="str">
-        <v>cloturee</v>
+        <v>bon_de_commande_envoye</v>
       </c>
       <c r="C47" t="str">
-        <v>Cloturee</v>
+        <v>BdC envoye au fournisseur</v>
       </c>
       <c r="D47" t="str">
-        <v>-</v>
+        <v>logistique</v>
       </c>
       <c r="E47" t="str">
-        <v>-</v>
+        <v>ar_recu</v>
       </c>
       <c r="F47" t="str">
-        <v>-</v>
+        <v>AR recu</v>
       </c>
       <c r="G47" t="str">
-        <v>terminal</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B48" t="str">
-        <v>abandonnee</v>
+        <v>ar_recu</v>
       </c>
       <c r="C48" t="str">
-        <v>Annulee</v>
+        <v>Accuse reception fournisseur</v>
       </c>
       <c r="D48" t="str">
+        <v>logistique</v>
+      </c>
+      <c r="E48" t="str">
+        <v>commande_livree</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Marquer livre</v>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>5</v>
+      </c>
+      <c r="B49" t="str">
+        <v>commande_livree</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Materiel recu chez nous</v>
+      </c>
+      <c r="D49" t="str">
+        <v>logistique</v>
+      </c>
+      <c r="E49" t="str">
+        <v>commande_distribuee</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Distribuer au technicien</v>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>6</v>
+      </c>
+      <c r="B50" t="str">
+        <v>commande_distribuee</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Remis au technicien (terminal)</v>
+      </c>
+      <c r="D50" t="str">
         <v>-</v>
       </c>
-      <c r="E48" t="str">
+      <c r="E50" t="str">
         <v>-</v>
       </c>
-      <c r="F48" t="str">
+      <c r="F50" t="str">
         <v>-</v>
       </c>
-      <c r="G48" t="str">
+      <c r="G50" t="str">
         <v>terminal</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
+    <row r="51">
+      <c r="A51">
+        <v>7</v>
+      </c>
+      <c r="B51" t="str">
+        <v>refusee</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Refusee par coordinateur</v>
+      </c>
+      <c r="D51" t="str">
+        <v>-</v>
+      </c>
+      <c r="E51" t="str">
+        <v>-</v>
+      </c>
+      <c r="F51" t="str">
+        <v>-</v>
+      </c>
+      <c r="G51" t="str">
+        <v>terminal - notif demandeur avec motif</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
         <v>### 5. SOUS-TACHES (uniquement si demande genere multi-taches) ###</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="str">
+    <row r="54">
+      <c r="A54" t="str">
         <v>#</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B54" t="str">
         <v>Prestation</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C54" t="str">
         <v>Sous-tache</v>
       </c>
-      <c r="D51" t="str">
+      <c r="D54" t="str">
         <v>Service cible</v>
       </c>
-      <c r="E51" t="str">
+      <c r="E54" t="str">
         <v>Affectation</v>
       </c>
-      <c r="F51" t="str">
+      <c r="F54" t="str">
         <v>Validateur N1</v>
       </c>
-      <c r="G51" t="str">
+      <c r="G54" t="str">
         <v>Duree</v>
       </c>
-      <c r="H51" t="str">
+      <c r="H54" t="str">
         <v>Ordre</v>
       </c>
-      <c r="I51" t="str">
+      <c r="I54" t="str">
         <v>Parallele ?</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52">
+    <row r="55">
+      <c r="A55">
         <v>1</v>
       </c>
-      <c r="B52" t="str">
-        <v/>
-      </c>
-      <c r="C52" t="str">
-        <v/>
-      </c>
-      <c r="D52" t="str">
-        <v/>
-      </c>
-      <c r="E52" t="str">
-        <v/>
-      </c>
-      <c r="F52" t="str">
-        <v/>
-      </c>
-      <c r="G52" t="str">
-        <v/>
-      </c>
-      <c r="H52">
+      <c r="B55" t="str">
+        <v/>
+      </c>
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55">
         <v>0</v>
       </c>
-      <c r="I52" t="str">
-        <v>OUI</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53">
+      <c r="I55" t="str">
+        <v>OUI</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
         <v>2</v>
       </c>
-      <c r="B53" t="str">
-        <v/>
-      </c>
-      <c r="C53" t="str">
-        <v/>
-      </c>
-      <c r="D53" t="str">
-        <v/>
-      </c>
-      <c r="E53" t="str">
-        <v/>
-      </c>
-      <c r="F53" t="str">
-        <v/>
-      </c>
-      <c r="G53" t="str">
-        <v/>
-      </c>
-      <c r="H53">
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v/>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56">
         <v>0</v>
       </c>
-      <c r="I53" t="str">
-        <v>OUI</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54">
+      <c r="I56" t="str">
+        <v>OUI</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
         <v>3</v>
       </c>
-      <c r="B54" t="str">
-        <v/>
-      </c>
-      <c r="C54" t="str">
-        <v/>
-      </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
-      <c r="E54" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
-        <v/>
-      </c>
-      <c r="G54" t="str">
-        <v/>
-      </c>
-      <c r="H54">
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57">
         <v>0</v>
       </c>
-      <c r="I54" t="str">
-        <v>OUI</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
+      <c r="I57" t="str">
+        <v>OUI</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
         <v>### 6. NOTIFICATIONS ###</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="str">
+    <row r="60">
+      <c r="A60" t="str">
         <v>#</v>
       </c>
-      <c r="B57" t="str">
+      <c r="B60" t="str">
         <v>Evenement</v>
       </c>
-      <c r="C57" t="str">
+      <c r="C60" t="str">
         <v>Destinataire(s)</v>
       </c>
-      <c r="D57" t="str">
+      <c r="D60" t="str">
         <v>Canal</v>
       </c>
-      <c r="E57" t="str">
+      <c r="E60" t="str">
         <v>Message</v>
       </c>
-      <c r="F57" t="str">
+      <c r="F60" t="str">
         <v>Priorite</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>1</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Demande soumise</v>
-      </c>
-      <c r="C58" t="str">
-        <v/>
-      </c>
-      <c r="D58" t="str">
-        <v>in-app</v>
-      </c>
-      <c r="E58" t="str">
-        <v/>
-      </c>
-      <c r="F58" t="str">
-        <v>normale</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59">
-        <v>2</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Affectation</v>
-      </c>
-      <c r="C59" t="str">
-        <v/>
-      </c>
-      <c r="D59" t="str">
-        <v>in-app</v>
-      </c>
-      <c r="E59" t="str">
-        <v/>
-      </c>
-      <c r="F59" t="str">
-        <v>normale</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60">
-        <v>3</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Demande validation</v>
-      </c>
-      <c r="C60" t="str">
-        <v/>
-      </c>
-      <c r="D60" t="str">
-        <v>in-app</v>
-      </c>
-      <c r="E60" t="str">
-        <v/>
-      </c>
-      <c r="F60" t="str">
-        <v>haute</v>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B61" t="str">
-        <v>Complement demande</v>
+        <v>Demande soumise</v>
       </c>
       <c r="C61" t="str">
-        <v/>
+        <v>Sylvain ANTZ</v>
       </c>
       <c r="D61" t="str">
         <v>in-app</v>
       </c>
       <c r="E61" t="str">
-        <v/>
+        <v>Nouvelle demande materiel de &lt;demandeur&gt; - &lt;N lignes&gt; articles</v>
       </c>
       <c r="F61" t="str">
         <v>haute</v>
@@ -9518,19 +9527,19 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B62" t="str">
-        <v>Validee / Refusee</v>
+        <v>Validee</v>
       </c>
       <c r="C62" t="str">
-        <v/>
+        <v>demandeur + logistique</v>
       </c>
       <c r="D62" t="str">
         <v>in-app</v>
       </c>
       <c r="E62" t="str">
-        <v/>
+        <v>Votre demande materiel est validee, en cours de commande</v>
       </c>
       <c r="F62" t="str">
         <v>normale</v>
@@ -9538,55 +9547,82 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B63" t="str">
-        <v>Cloturee</v>
+        <v>Refusee</v>
       </c>
       <c r="C63" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="D63" t="str">
         <v>in-app</v>
       </c>
       <c r="E63" t="str">
-        <v/>
+        <v>Votre demande materiel a ete refusee : &lt;motif&gt;</v>
       </c>
       <c r="F63" t="str">
-        <v>normale</v>
+        <v>haute</v>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B64" t="str">
-        <v>SLA depasse</v>
+        <v>BdC envoye</v>
       </c>
       <c r="C64" t="str">
-        <v/>
+        <v>demandeur</v>
       </c>
       <c r="D64" t="str">
         <v>in-app</v>
       </c>
       <c r="E64" t="str">
-        <v/>
+        <v>Votre commande a ete passee aupres du fournisseur</v>
       </c>
       <c r="F64" t="str">
-        <v>urgente</v>
+        <v>normale</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="str">
-        <v/>
+      <c r="A65">
+        <v>5</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Livree</v>
+      </c>
+      <c r="C65" t="str">
+        <v>demandeur</v>
+      </c>
+      <c r="D65" t="str">
+        <v>in-app</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Votre materiel est arrive, viens le retirer</v>
+      </c>
+      <c r="F65" t="str">
+        <v>haute</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="str">
-        <v># Note</v>
+      <c r="A66">
+        <v>6</v>
       </c>
       <c r="B66" t="str">
-        <v>Le commentaire de tache est deja gere par le trigger BE-010 (notif assigne+manager+demandeur). Inutile de le re-declarer.</v>
+        <v>Distribuee</v>
+      </c>
+      <c r="C66" t="str">
+        <v>demandeur</v>
+      </c>
+      <c r="D66" t="str">
+        <v>in-app</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Materiel remis - merci de confirmer reception</v>
+      </c>
+      <c r="F66" t="str">
+        <v>normale</v>
       </c>
     </row>
     <row r="67">
@@ -9596,60 +9632,45 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>### 7. KPI DASHBOARD ###</v>
+        <v># Note</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Le commentaire de tache est deja gere par le trigger BE-010 (notif assigne+manager+demandeur). Inutile de le re-declarer.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>### 7. KPI DASHBOARD ###</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
         <v>#</v>
       </c>
-      <c r="B69" t="str">
+      <c r="B71" t="str">
         <v>KPI (label)</v>
       </c>
-      <c r="C69" t="str">
+      <c r="C71" t="str">
         <v>Formule</v>
       </c>
-      <c r="D69" t="str">
+      <c r="D71" t="str">
         <v>Couleur</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70">
-        <v>1</v>
-      </c>
-      <c r="B70" t="str">
-        <v>Total actives</v>
-      </c>
-      <c r="C70" t="str">
-        <v>count(status NOT IN terminaux)</v>
-      </c>
-      <c r="D70" t="str">
-        <v>neutre</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71">
-        <v>2</v>
-      </c>
-      <c r="B71" t="str">
-        <v>En retard</v>
-      </c>
-      <c r="C71" t="str">
-        <v>count(due_date &lt; today AND active)</v>
-      </c>
-      <c r="D71" t="str">
-        <v>rouge</v>
       </c>
     </row>
     <row r="72">
       <c r="A72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B72" t="str">
-        <v>A valider</v>
+        <v>Demandes en attente validation</v>
       </c>
       <c r="C72" t="str">
-        <v>count(status=a_valider)</v>
+        <v>count(status=en_attente_validation)</v>
       </c>
       <c r="D72" t="str">
         <v>ambre</v>
@@ -9657,81 +9678,90 @@
     </row>
     <row r="73">
       <c r="A73">
+        <v>2</v>
+      </c>
+      <c r="B73" t="str">
+        <v>En cours de commande</v>
+      </c>
+      <c r="C73" t="str">
+        <v>count(status IN (demande_de_devis, bon_de_commande_envoye, ar_recu))</v>
+      </c>
+      <c r="D73" t="str">
+        <v>bleu</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>3</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Livrees a distribuer</v>
+      </c>
+      <c r="C74" t="str">
+        <v>count(status=commande_livree)</v>
+      </c>
+      <c r="D74" t="str">
+        <v>vert</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
         <v>4</v>
       </c>
-      <c r="B73" t="str">
-        <v>Non assignees</v>
-      </c>
-      <c r="C73" t="str">
-        <v>count(assignee_id IS NULL AND active)</v>
-      </c>
-      <c r="D73" t="str">
-        <v>violet</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="str">
-        <v># Filtres souhaites</v>
-      </c>
       <c r="B75" t="str">
-        <v>Active ?</v>
+        <v>Refusees ce mois</v>
       </c>
       <c r="C75" t="str">
-        <v>Notes</v>
+        <v>count(status=refusee AND month=current)</v>
+      </c>
+      <c r="D75" t="str">
+        <v>rouge</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="str">
-        <v>Recherche libre</v>
+      <c r="A76">
+        <v>5</v>
       </c>
       <c r="B76" t="str">
-        <v>OUI</v>
+        <v>Total articles commandes ce mois</v>
       </c>
       <c r="C76" t="str">
-        <v>titre / numero</v>
+        <v>sum(quantite) sur ce mois</v>
+      </c>
+      <c r="D76" t="str">
+        <v>neutre</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Statut</v>
-      </c>
-      <c r="B77" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="C77" t="str">
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Demandeur</v>
+        <v># Filtres souhaites</v>
       </c>
       <c r="B78" t="str">
-        <v>OUI</v>
+        <v>Active ?</v>
       </c>
       <c r="C78" t="str">
-        <v/>
+        <v>Notes</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Assigne</v>
+        <v>Recherche libre</v>
       </c>
       <c r="B79" t="str">
         <v>OUI</v>
       </c>
       <c r="C79" t="str">
-        <v/>
+        <v>titre / numero</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>En retard (toggle)</v>
+        <v>Statut</v>
       </c>
       <c r="B80" t="str">
         <v>OUI</v>
@@ -9742,10 +9772,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Prestation</v>
+        <v>Demandeur</v>
       </c>
       <c r="B81" t="str">
-        <v/>
+        <v>OUI</v>
       </c>
       <c r="C81" t="str">
         <v/>
@@ -9753,10 +9783,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Filtre metier 1</v>
+        <v>Assigne</v>
       </c>
       <c r="B82" t="str">
-        <v/>
+        <v>OUI</v>
       </c>
       <c r="C82" t="str">
         <v/>
@@ -9764,124 +9794,79 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
+        <v>En retard (toggle)</v>
+      </c>
+      <c r="B83" t="str">
+        <v>OUI</v>
+      </c>
+      <c r="C83" t="str">
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>### 8. PERMISSIONS ###</v>
+        <v>Prestation</v>
+      </c>
+      <c r="B84" t="str">
+        <v/>
+      </c>
+      <c r="C84" t="str">
+        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Action</v>
+        <v>Filtre metier 1</v>
       </c>
       <c r="B85" t="str">
-        <v>Demandeur</v>
+        <v/>
       </c>
       <c r="C85" t="str">
-        <v>Executant/Cible</v>
-      </c>
-      <c r="D85" t="str">
-        <v>Manager service</v>
-      </c>
-      <c r="E85" t="str">
-        <v>Validateur N1</v>
-      </c>
-      <c r="F85" t="str">
-        <v>Validateur N2</v>
-      </c>
-      <c r="G85" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="H85" t="str">
-        <v>Autre</v>
+        <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Creer demande</v>
-      </c>
-      <c r="B86" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="C86" t="str">
-        <v/>
-      </c>
-      <c r="D86" t="str">
-        <v/>
-      </c>
-      <c r="E86" t="str">
-        <v/>
-      </c>
-      <c r="F86" t="str">
-        <v/>
-      </c>
-      <c r="G86" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="H86" t="str">
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Voir ses demandes</v>
-      </c>
-      <c r="B87" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="C87" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="D87" t="str">
-        <v/>
-      </c>
-      <c r="E87" t="str">
-        <v/>
-      </c>
-      <c r="F87" t="str">
-        <v/>
-      </c>
-      <c r="G87" t="str">
-        <v>OUI</v>
-      </c>
-      <c r="H87" t="str">
-        <v/>
+        <v>### 8. PERMISSIONS ###</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Voir TOUTES</v>
+        <v>Action</v>
       </c>
       <c r="B88" t="str">
-        <v/>
+        <v>Demandeur</v>
       </c>
       <c r="C88" t="str">
-        <v/>
+        <v>Executant/Cible</v>
       </c>
       <c r="D88" t="str">
-        <v/>
+        <v>Manager service</v>
       </c>
       <c r="E88" t="str">
-        <v/>
+        <v>Validateur N1</v>
       </c>
       <c r="F88" t="str">
-        <v/>
+        <v>Validateur N2</v>
       </c>
       <c r="G88" t="str">
-        <v>OUI</v>
+        <v>Admin</v>
       </c>
       <c r="H88" t="str">
-        <v/>
+        <v>Autre</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Affecter</v>
+        <v>Creer demande</v>
       </c>
       <c r="B89" t="str">
-        <v/>
+        <v>OUI (technicien maintenance)</v>
       </c>
       <c r="C89" t="str">
         <v/>
@@ -9904,10 +9889,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Reaffecter</v>
+        <v>Voir ses demandes</v>
       </c>
       <c r="B90" t="str">
-        <v/>
+        <v>OUI</v>
       </c>
       <c r="C90" t="str">
         <v/>
@@ -9930,10 +9915,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Annuler</v>
+        <v>Voir TOUTES</v>
       </c>
       <c r="B91" t="str">
-        <v>sienne</v>
+        <v/>
       </c>
       <c r="C91" t="str">
         <v/>
@@ -9951,12 +9936,12 @@
         <v>OUI</v>
       </c>
       <c r="H91" t="str">
-        <v/>
+        <v>Sylvain + logistique</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Valider N1</v>
+        <v>Valider/Refuser</v>
       </c>
       <c r="B92" t="str">
         <v/>
@@ -9968,7 +9953,7 @@
         <v/>
       </c>
       <c r="E92" t="str">
-        <v>OUI</v>
+        <v/>
       </c>
       <c r="F92" t="str">
         <v/>
@@ -9977,12 +9962,12 @@
         <v>OUI</v>
       </c>
       <c r="H92" t="str">
-        <v/>
+        <v>Sylvain ANTZ</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Valider N2</v>
+        <v>Faire avancer etat commande</v>
       </c>
       <c r="B93" t="str">
         <v/>
@@ -9997,61 +9982,76 @@
         <v/>
       </c>
       <c r="F93" t="str">
-        <v>OUI</v>
+        <v/>
       </c>
       <c r="G93" t="str">
         <v>OUI</v>
       </c>
       <c r="H93" t="str">
-        <v/>
+        <v>logistique</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
+        <v>Annuler une demande</v>
+      </c>
+      <c r="B94" t="str">
+        <v>la sienne (avant validation)</v>
+      </c>
+      <c r="C94" t="str">
+        <v/>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+      <c r="G94" t="str">
+        <v>OUI</v>
+      </c>
+      <c r="H94" t="str">
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>### 9. HUB PROJET / DOSSIER (si applicable) ###</v>
+        <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Champ</v>
-      </c>
-      <c r="B96" t="str">
-        <v>Valeur</v>
-      </c>
-      <c r="C96" t="str">
-        <v>Aide</v>
+        <v>### 9. HUB PROJET / DOSSIER (si applicable) ###</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Hub active ?</v>
+        <v>Champ</v>
       </c>
       <c r="B97" t="str">
-        <v/>
+        <v>Valeur</v>
       </c>
       <c r="C97" t="str">
-        <v>OUI / NON</v>
+        <v>Aide</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Concept</v>
+        <v>Hub active ?</v>
       </c>
       <c r="B98" t="str">
-        <v/>
+        <v>NON</v>
       </c>
       <c r="C98" t="str">
-        <v>ex. dossier client, projet R&amp;D, audit</v>
+        <v>chaque demande est independante</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Nom entite</v>
+        <v>Concept</v>
       </c>
       <c r="B99" t="str">
         <v/>
@@ -10062,196 +10062,181 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Code/identifiant</v>
+        <v>Nom entite</v>
       </c>
       <c r="B100" t="str">
         <v/>
       </c>
       <c r="C100" t="str">
-        <v>format</v>
+        <v/>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Onglets souhaites</v>
+        <v>Code/identifiant</v>
       </c>
       <c r="B101" t="str">
         <v/>
       </c>
       <c r="C101" t="str">
-        <v>Fiche / Taches / Timeline / Discussions / Fichiers</v>
+        <v/>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Visibilite</v>
+        <v>Onglets</v>
       </c>
       <c r="B102" t="str">
         <v/>
       </c>
       <c r="C102" t="str">
-        <v>qui peut lire / ecrire</v>
+        <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
+        <v>Visibilite</v>
+      </c>
+      <c r="B103" t="str">
+        <v/>
+      </c>
+      <c r="C103" t="str">
         <v/>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>### 10. INTEGRATIONS EXTERNES ###</v>
+        <v/>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Outil</v>
-      </c>
-      <c r="B105" t="str">
-        <v>Pour quoi ?</v>
-      </c>
-      <c r="C105" t="str">
-        <v>Sens</v>
-      </c>
-      <c r="D105" t="str">
-        <v>Statut</v>
-      </c>
-      <c r="E105" t="str">
-        <v>Priorite</v>
+        <v>### 10. INTEGRATIONS EXTERNES ###</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Lucca</v>
+        <v>Outil</v>
       </c>
       <c r="B106" t="str">
-        <v/>
+        <v>Pour quoi ?</v>
       </c>
       <c r="C106" t="str">
-        <v/>
+        <v>Sens</v>
       </c>
       <c r="D106" t="str">
-        <v/>
+        <v>Statut</v>
       </c>
       <c r="E106" t="str">
-        <v/>
+        <v>Priorite</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Yooz</v>
+        <v>Divalto</v>
       </c>
       <c r="B107" t="str">
-        <v/>
+        <v>referentiel articles + creation BdC</v>
       </c>
       <c r="C107" t="str">
-        <v/>
+        <v>lecture+ecriture</v>
       </c>
       <c r="D107" t="str">
-        <v/>
+        <v>partiel</v>
       </c>
       <c r="E107" t="str">
-        <v/>
+        <v>haute</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Pipedrive</v>
+        <v>Yooz</v>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>rapprochement facture fournisseur</v>
       </c>
       <c r="C108" t="str">
-        <v/>
+        <v>lecture</v>
       </c>
       <c r="D108" t="str">
-        <v/>
+        <v>a faire</v>
       </c>
       <c r="E108" t="str">
-        <v/>
+        <v>normale</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Divalto</v>
-      </c>
-      <c r="B109" t="str">
-        <v/>
-      </c>
-      <c r="C109" t="str">
-        <v/>
-      </c>
-      <c r="D109" t="str">
-        <v/>
-      </c>
-      <c r="E109" t="str">
         <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>SharePoint</v>
-      </c>
-      <c r="B110" t="str">
-        <v/>
-      </c>
-      <c r="C110" t="str">
-        <v/>
-      </c>
-      <c r="D110" t="str">
-        <v/>
-      </c>
-      <c r="E110" t="str">
-        <v/>
+        <v>### 11. QUESTIONS OUVERTES ###</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v/>
+        <v>#</v>
       </c>
       <c r="B111" t="str">
-        <v/>
+        <v>Question</v>
       </c>
       <c r="C111" t="str">
-        <v/>
+        <v>Importance</v>
       </c>
       <c r="D111" t="str">
-        <v/>
-      </c>
-      <c r="E111" t="str">
-        <v/>
+        <v>Reponse</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="str">
+      <c r="A112">
+        <v>1</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Le coordinateur Sylvain a-t-il un suppleant si absent ?</v>
+      </c>
+      <c r="C112" t="str">
+        <v>bloquant</v>
+      </c>
+      <c r="D112" t="str">
         <v/>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="str">
-        <v>### 11. QUESTIONS OUVERTES ###</v>
+      <c r="A113">
+        <v>2</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Refus : doit-on imposer un motif ? template de motifs ?</v>
+      </c>
+      <c r="C113" t="str">
+        <v>normal</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="str">
-        <v>#</v>
+      <c r="A114">
+        <v>3</v>
       </c>
       <c r="B114" t="str">
-        <v>Question</v>
+        <v>Articles : on garde le catalogue Divalto comme referentiel ou on stocke localement ?</v>
       </c>
       <c r="C114" t="str">
-        <v>Importance</v>
+        <v>normal</v>
       </c>
       <c r="D114" t="str">
-        <v>Reponse</v>
+        <v/>
       </c>
     </row>
     <row r="115">
       <c r="A115">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B115" t="str">
-        <v/>
+        <v>Limite budgetaire par demande (validation N2 si &gt; X EUR) ?</v>
       </c>
       <c r="C115" t="str">
         <v>normal</v>
@@ -10262,13 +10247,13 @@
     </row>
     <row r="116">
       <c r="A116">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B116" t="str">
-        <v/>
+        <v>Reset a zero des anciennes demandes en prod ?</v>
       </c>
       <c r="C116" t="str">
-        <v>normal</v>
+        <v>bloquant</v>
       </c>
       <c r="D116" t="str">
         <v/>
@@ -10276,10 +10261,10 @@
     </row>
     <row r="117">
       <c r="A117">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B117" t="str">
-        <v/>
+        <v>Le bouton "Distribuer" ferme la demande ou il y a une etape "confirmation reception technicien" ?</v>
       </c>
       <c r="C117" t="str">
         <v>normal</v>
@@ -10288,37 +10273,9 @@
         <v/>
       </c>
     </row>
-    <row r="118">
-      <c r="A118">
-        <v>4</v>
-      </c>
-      <c r="B118" t="str">
-        <v/>
-      </c>
-      <c r="C118" t="str">
-        <v>normal</v>
-      </c>
-      <c r="D118" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119">
-        <v>5</v>
-      </c>
-      <c r="B119" t="str">
-        <v/>
-      </c>
-      <c r="C119" t="str">
-        <v>normal</v>
-      </c>
-      <c r="D119" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I119"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I117"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>